<commit_message>
Atualiza planilha de colaboradores (nova colaboradora) e ajustes locais (porta 8080)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Planilha de colaboradores.xlsx
+++ b/Planilha de colaboradores.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02546682d8504731/Área de Trabalho/Mateus - RH/Colaboradores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="919" documentId="8_{3A3BF5FC-571E-435F-BABF-BF226CCBF53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EE9CC57-EB6B-4DFD-9D7B-2A9C2653C263}"/>
+  <xr:revisionPtr revIDLastSave="923" documentId="8_{3A3BF5FC-571E-435F-BABF-BF226CCBF53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CE6527C-8713-4186-BF73-BFB70DFBD919}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CFC07945-D250-4F6F-B900-FCF791F3ED89}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
   <si>
     <t>Colaboradores</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>Deborah Sztajin</t>
+  </si>
+  <si>
+    <t>Mariana Borges</t>
   </si>
 </sst>
 </file>
@@ -574,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7546B69-D4A2-4D9E-ABFD-0C0FA78CC7D2}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5546875" style="1" customWidth="1"/>
@@ -760,35 +763,35 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>15</v>
+        <v>29</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="C17" s="3">
-        <v>95</v>
+        <v>223</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="3">
-        <v>131</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="3">
-        <v>215</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -796,43 +799,43 @@
         <v>31</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="3">
-        <v>27</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>19</v>
+        <v>31</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="C21" s="3">
-        <v>85</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>20</v>
+        <v>28</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="C22" s="3">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3">
-        <v>13</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -840,48 +843,55 @@
         <v>29</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C24" s="3">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="3">
-        <v>117</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" s="3">
-        <v>165</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B28" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C28" s="3">
         <v>35</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B28"/>
-      <c r="C28"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B29"/>
@@ -890,6 +900,10 @@
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B30"/>
       <c r="C30"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B31"/>
+      <c r="C31"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Inclui Pamela Moreira na planilha de colaboradores (COMERCIAL).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Planilha de colaboradores.xlsx
+++ b/Planilha de colaboradores.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02546682d8504731/Área de Trabalho/Mateus - RH/Colaboradores/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mateus\.cursor\projects\bitrix-exporter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="923" documentId="8_{3A3BF5FC-571E-435F-BABF-BF226CCBF53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CE6527C-8713-4186-BF73-BFB70DFBD919}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8656D8C-F728-4F86-AFC5-5230DA74F306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CFC07945-D250-4F6F-B900-FCF791F3ED89}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
   <si>
     <t>Colaboradores</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>Mariana Borges</t>
+  </si>
+  <si>
+    <t>Pamela Moreira</t>
   </si>
 </sst>
 </file>
@@ -274,10 +277,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -577,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7546B69-D4A2-4D9E-ABFD-0C0FA78CC7D2}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5546875" style="1" customWidth="1"/>
@@ -807,46 +806,46 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C21" s="3">
-        <v>27</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>19</v>
+        <v>31</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="C22" s="3">
-        <v>85</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>20</v>
+        <v>28</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="C23" s="3">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="3">
-        <v>13</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -854,48 +853,55 @@
         <v>29</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C25" s="3">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" s="3">
-        <v>117</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27" s="3">
-        <v>165</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B29" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C29" s="3">
         <v>35</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B29"/>
-      <c r="C29"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B30"/>
@@ -904,6 +910,10 @@
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B31"/>
       <c r="C31"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B32"/>
+      <c r="C32"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>